<commit_message>
First real commit. Got framework to fill with real values
</commit_message>
<xml_diff>
--- a/data/blocages.xlsx
+++ b/data/blocages.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Personne 02</t>
+          <t>Personne 01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -476,42 +476,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Samedi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Personne 03</t>
+          <t>Personne 02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Samedi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -526,21 +526,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -556,16 +556,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -576,17 +576,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>24:00</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -596,47 +596,47 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Personne 12</t>
+          <t>Personne 08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Samedi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Personne 17</t>
+          <t>Personne 13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -646,7 +646,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Personne 19</t>
+          <t>Personne 14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -656,12 +656,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>24:00</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -671,47 +671,47 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Personne 19</t>
+          <t>Personne 14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Personne 20</t>
+          <t>Personne 17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -721,51 +721,51 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Personne 21</t>
+          <t>Personne 17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Personne 21</t>
+          <t>Personne 22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +776,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -796,22 +796,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Personne 22</t>
+          <t>Personne 24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -826,42 +826,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Personne 24</t>
+          <t>Personne 25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -871,12 +871,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personne 26</t>
+          <t>Personne 28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -886,32 +886,32 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Personne 27</t>
+          <t>Personne 36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -921,7 +921,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Personne 27</t>
+          <t>Personne 38</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>24:00</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -946,22 +946,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Personne 30</t>
+          <t>Personne 38</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Vendredi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>24:00</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -971,22 +971,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Personne 30</t>
+          <t>Personne 39</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -996,12 +996,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Personne 32</t>
+          <t>Personne 40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Samedi</t>
+          <t>Mardi</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1021,12 +1021,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Personne 32</t>
+          <t>Personne 41</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1036,47 +1036,47 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Personne 33</t>
+          <t>Personne 41</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Personne 33</t>
+          <t>Personne 43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1096,22 +1096,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Personne 39</t>
+          <t>Personne 46</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1121,22 +1121,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Personne 39</t>
+          <t>Personne 48</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1146,22 +1146,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Personne 40</t>
+          <t>Personne 50</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Mardi</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1171,12 +1171,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Personne 43</t>
+          <t>Personne 51</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1196,47 +1196,47 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Personne 43</t>
+          <t>Personne 53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Personne 45</t>
+          <t>Personne 53</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1246,47 +1246,47 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Personne 45</t>
+          <t>Personne 55</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Personne 59</t>
+          <t>Personne 56</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Mardi</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1296,7 +1296,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Personne 61</t>
+          <t>Personne 59</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1306,57 +1306,57 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Personne 62</t>
+          <t>Personne 59</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Vendredi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Personne 62</t>
+          <t>Personne 69</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1366,181 +1366,6 @@
       </c>
       <c r="E38" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Personne 65</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Mercredi</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Personne 65</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Lundi</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Personne 66</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Dimanche</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Personne 67</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Mercredi</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Personne 67</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Vendredi</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Personne 68</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Jeudi</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Personne 68</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Mercredi</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First beta-planning for Mardi with all constraints EXCEPT concerts
</commit_message>
<xml_diff>
--- a/data/blocages.xlsx
+++ b/data/blocages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FEA98B-A0CC-42CD-98E0-57FDABD73BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F5F8C0-B092-4573-A63D-67748C5F6611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mardi" sheetId="1" r:id="rId1"/>
@@ -1183,30 +1183,30 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>

</xml_diff>

<commit_message>
Grille horaire with printer-friendly layout
</commit_message>
<xml_diff>
--- a/data/blocages.xlsx
+++ b/data/blocages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sschies1\_code\1.09_VScode\06_VoeuxConcerts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C761906-A988-4ABE-9FED-23B989B7BA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86924202-825D-41AD-815F-A4E20490BECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="1480" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mardi" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
   <externalReferences>
     <externalReference r:id="rId8"/>
   </externalReferences>
-  <calcPr calcId="191029" iterate="1" iterateCount="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1627,6 +1627,16 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
+        <row r="1">
+          <cell r="B1"/>
+          <cell r="E1"/>
+          <cell r="F1"/>
+        </row>
+        <row r="2">
+          <cell r="B2"/>
+          <cell r="E2"/>
+          <cell r="F2"/>
+        </row>
         <row r="3">
           <cell r="B3" t="str">
             <v>In</v>
@@ -2390,6 +2400,7 @@
           <cell r="B72" t="b">
             <v>0</v>
           </cell>
+          <cell r="E72"/>
           <cell r="F72" t="str">
             <v>Michelle-Evy</v>
           </cell>
@@ -2618,6 +2629,7 @@
           <cell r="B93" t="b">
             <v>0</v>
           </cell>
+          <cell r="E93"/>
           <cell r="F93" t="str">
             <v>Ramón</v>
           </cell>
@@ -2632,6 +2644,11 @@
           <cell r="F94" t="str">
             <v>Robert</v>
           </cell>
+        </row>
+        <row r="95">
+          <cell r="B95"/>
+          <cell r="E95"/>
+          <cell r="F95"/>
         </row>
       </sheetData>
       <sheetData sheetId="1"/>

</xml_diff>